<commit_message>
NCR 피드백 최종반영: 사진D9:F17, 특기사항A18:F20, Sheet1삭제. Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ncr_template.xlsx
+++ b/ncr_template.xlsx
@@ -7,7 +7,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02.12.11" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -731,7 +730,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1138,6 +1137,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1857,29 +1859,32 @@
       <c r="I17" s="138" t="n"/>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="141" t="inlineStr">
+      <c r="A18" s="158" t="inlineStr">
         <is>
           <t>※특기사항</t>
         </is>
       </c>
       <c r="B18" s="123" t="n"/>
-      <c r="C18" s="124" t="n"/>
-      <c r="D18" s="136" t="n"/>
+      <c r="C18" s="123" t="n"/>
+      <c r="D18" s="123" t="n"/>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="124" t="n"/>
       <c r="G18" s="136" t="n"/>
       <c r="I18" s="138" t="n"/>
     </row>
     <row r="19" hidden="1" ht="18.75" customHeight="1">
       <c r="A19" s="134" t="n"/>
-      <c r="C19" s="135" t="n"/>
-      <c r="D19" s="136" t="n"/>
+      <c r="F19" s="135" t="n"/>
       <c r="G19" s="136" t="n"/>
       <c r="I19" s="138" t="n"/>
     </row>
     <row r="20" ht="0.75" customHeight="1" thickBot="1">
       <c r="A20" s="142" t="n"/>
       <c r="B20" s="118" t="n"/>
-      <c r="C20" s="143" t="n"/>
-      <c r="D20" s="136" t="n"/>
+      <c r="C20" s="118" t="n"/>
+      <c r="D20" s="118" t="n"/>
+      <c r="E20" s="118" t="n"/>
+      <c r="F20" s="143" t="n"/>
       <c r="G20" s="125" t="n"/>
       <c r="H20" s="126" t="n"/>
       <c r="I20" s="144" t="n"/>
@@ -2228,18 +2233,18 @@
     <mergeCell ref="I23:I25"/>
     <mergeCell ref="H37:H39"/>
     <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A2:C2"/>
     <mergeCell ref="B36:E36"/>
-    <mergeCell ref="A18:C20"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="D27:F35"/>
+    <mergeCell ref="D4:F4"/>
     <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A18:F20"/>
     <mergeCell ref="A27:C35"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D4:F4"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="H23:H25"/>
@@ -2247,7 +2252,6 @@
     <mergeCell ref="H27:H35"/>
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="A43:I43"/>
-    <mergeCell ref="D9:F20"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="D26:F26"/>
@@ -2256,6 +2260,7 @@
     <mergeCell ref="G3:I4"/>
     <mergeCell ref="G14:I20"/>
     <mergeCell ref="G23:G25"/>
+    <mergeCell ref="D9:F17"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="G27:G35"/>
     <mergeCell ref="G11:I11"/>
@@ -2277,56 +2282,4 @@
   <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A3:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
-  <cols>
-    <col width="14.109375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="3">
-      <c r="A3" s="26" t="n"/>
-      <c r="B3" s="26" t="n"/>
-      <c r="C3" s="26" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="26" t="n"/>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-    </row>
-    <row r="5" ht="26.25" customHeight="1">
-      <c r="A5" s="26" t="n"/>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">결 재 득 </t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="26" t="n"/>
-      <c r="B6" s="26" t="n"/>
-      <c r="C6" s="26" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="26" t="n"/>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="26" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="n"/>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
-</worksheet>
 </file>
</xml_diff>